<commit_message>
pre updating paper 1 to v2
</commit_message>
<xml_diff>
--- a/data/processed/ettehad_rr_bp_reduction_effects.xlsx
+++ b/data/processed/ettehad_rr_bp_reduction_effects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/ResolveToSaveLives/100MLives/Github/UW-RTSL-100MLives/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WHO-CVD/github/uw-who-cvdtargets/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{331CF8A5-94EE-488E-B7B7-4C4AC6851445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{061EE65F-335A-43A2-A5B6-944F3AB48A16}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="8_{331CF8A5-94EE-488E-B7B7-4C4AC6851445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1677BEB-9CFA-41E6-A963-AF5371A2E9DD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{ACAEEDB5-3BB2-45B3-B3BF-2A292CDA7EEB}"/>
   </bookViews>
@@ -305,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -366,6 +366,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="5" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -701,7 +702,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7FBF1AE-BCF8-40A0-B451-998C10F2396D}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.77734375" customWidth="1"/>
@@ -712,7 +713,7 @@
     <col min="7" max="7" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -735,7 +736,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
@@ -759,8 +760,12 @@
         <f>1-F2</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I2" s="28">
+        <f>+G2/E2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -784,8 +789,12 @@
         <f t="shared" ref="G3" si="1">1-F3</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I3" s="28">
+        <f t="shared" ref="I3:I41" si="2">+G3/E3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -809,8 +818,12 @@
         <f>1-F4</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I4" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -836,8 +849,12 @@
         <f>1-F5</f>
         <v>0.37750000000000006</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I5" s="28">
+        <f t="shared" si="2"/>
+        <v>2.2205882352941173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
@@ -860,11 +877,15 @@
         <v>0.59759999999999991</v>
       </c>
       <c r="G6" s="11">
-        <f t="shared" ref="G6:G9" si="2">1-F6</f>
+        <f t="shared" ref="G6:G9" si="3">1-F6</f>
         <v>0.40240000000000009</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I6" s="28">
+        <f t="shared" si="2"/>
+        <v>1.9803149606299213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>2</v>
       </c>
@@ -887,11 +908,15 @@
         <v>0.36453599999999997</v>
       </c>
       <c r="G7" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.63546400000000003</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I7" s="28">
+        <f t="shared" si="2"/>
+        <v>1.2364267480231619</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>2</v>
       </c>
@@ -914,11 +939,15 @@
         <v>0.22236695999999997</v>
       </c>
       <c r="G8" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.77763304</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I8" s="28">
+        <f t="shared" si="2"/>
+        <v>1.1053606119889687</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>2</v>
       </c>
@@ -941,11 +970,15 @@
         <v>0.13564384559999998</v>
       </c>
       <c r="G9" s="11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.86435615440000002</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I9" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0551975611493931</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
@@ -969,8 +1002,12 @@
         <f>1-F10</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I10" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
@@ -984,18 +1021,22 @@
         <v>0</v>
       </c>
       <c r="E11" s="11">
-        <f t="shared" ref="E11" si="3">1-D11</f>
+        <f t="shared" ref="E11" si="4">1-D11</f>
         <v>1</v>
       </c>
       <c r="F11" s="5">
         <v>0</v>
       </c>
       <c r="G11" s="11">
-        <f t="shared" ref="G11" si="4">1-F11</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G11" si="5">1-F11</f>
+        <v>1</v>
+      </c>
+      <c r="I11" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1019,8 +1060,12 @@
         <f>1-F12</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I12" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>11</v>
       </c>
@@ -1046,8 +1091,12 @@
         <f>1-F13</f>
         <v>0.43059999999999998</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I13" s="28">
+        <f t="shared" si="2"/>
+        <v>1.9572727272727275</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
@@ -1062,7 +1111,7 @@
         <v>0.50700000000000001</v>
       </c>
       <c r="E14" s="11">
-        <f t="shared" ref="E14:E17" si="5">1-D14</f>
+        <f t="shared" ref="E14:E17" si="6">1-D14</f>
         <v>0.49299999999999999</v>
       </c>
       <c r="F14" s="6">
@@ -1070,11 +1119,15 @@
         <v>0.37010999999999999</v>
       </c>
       <c r="G14" s="11">
-        <f t="shared" ref="G14:G17" si="6">1-F14</f>
+        <f t="shared" ref="G14:G17" si="7">1-F14</f>
         <v>0.62989000000000006</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I14" s="28">
+        <f t="shared" si="2"/>
+        <v>1.2776673427991887</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>11</v>
       </c>
@@ -1089,7 +1142,7 @@
         <v>0.35489999999999999</v>
       </c>
       <c r="E15" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.64510000000000001</v>
       </c>
       <c r="F15" s="6">
@@ -1097,11 +1150,15 @@
         <v>0.259077</v>
       </c>
       <c r="G15" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.740923</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I15" s="28">
+        <f t="shared" si="2"/>
+        <v>1.1485397612773214</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>11</v>
       </c>
@@ -1116,7 +1173,7 @@
         <v>0.24842999999999996</v>
       </c>
       <c r="E16" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.75157000000000007</v>
       </c>
       <c r="F16" s="6">
@@ -1124,11 +1181,15 @@
         <v>0.18135389999999996</v>
       </c>
       <c r="G16" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.81864610000000004</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I16" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0892479742405896</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>11</v>
       </c>
@@ -1143,7 +1204,7 @@
         <v>0.17390099999999997</v>
       </c>
       <c r="E17" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.82609900000000003</v>
       </c>
       <c r="F17" s="6">
@@ -1151,11 +1212,15 @@
         <v>0.12694772999999998</v>
       </c>
       <c r="G17" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.87305227000000007</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I17" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0568373403187754</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>12</v>
       </c>
@@ -1179,8 +1244,12 @@
         <f>1-F18</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I18" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
@@ -1194,18 +1263,22 @@
         <v>0</v>
       </c>
       <c r="E19" s="11">
-        <f t="shared" ref="E19" si="7">1-D19</f>
+        <f t="shared" ref="E19" si="8">1-D19</f>
         <v>1</v>
       </c>
       <c r="F19" s="5">
         <v>0</v>
       </c>
       <c r="G19" s="11">
-        <f t="shared" ref="G19" si="8">1-F19</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G19" si="9">1-F19</f>
+        <v>1</v>
+      </c>
+      <c r="I19" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
@@ -1229,8 +1302,12 @@
         <f>1-F20</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I20" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>12</v>
       </c>
@@ -1256,8 +1333,12 @@
         <f>1-F21</f>
         <v>0.29599999999999993</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I21" s="28">
+        <f t="shared" si="2"/>
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>12</v>
       </c>
@@ -1272,7 +1353,7 @@
         <v>0.67200000000000004</v>
       </c>
       <c r="E22" s="11">
-        <f t="shared" ref="E22:E25" si="9">1-D22</f>
+        <f t="shared" ref="E22:E25" si="10">1-D22</f>
         <v>0.32799999999999996</v>
       </c>
       <c r="F22" s="6">
@@ -1280,11 +1361,15 @@
         <v>0.59136</v>
       </c>
       <c r="G22" s="11">
-        <f t="shared" ref="G22:G25" si="10">1-F22</f>
+        <f t="shared" ref="G22:G25" si="11">1-F22</f>
         <v>0.40864</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I22" s="28">
+        <f t="shared" si="2"/>
+        <v>1.2458536585365856</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
@@ -1299,7 +1384,7 @@
         <v>0.55103999999999997</v>
       </c>
       <c r="E23" s="11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.44896000000000003</v>
       </c>
       <c r="F23" s="6">
@@ -1307,11 +1392,15 @@
         <v>0.48491519999999999</v>
       </c>
       <c r="G23" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.51508480000000001</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I23" s="28">
+        <f t="shared" si="2"/>
+        <v>1.1472843905915895</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>12</v>
       </c>
@@ -1326,7 +1415,7 @@
         <v>0.45185279999999994</v>
       </c>
       <c r="E24" s="11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.54814720000000006</v>
       </c>
       <c r="F24" s="6">
@@ -1334,11 +1423,15 @@
         <v>0.39763046399999996</v>
       </c>
       <c r="G24" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.60236953600000009</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I24" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0989192975901365</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>12</v>
       </c>
@@ -1353,7 +1446,7 @@
         <v>0.37051929599999989</v>
       </c>
       <c r="E25" s="11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.62948070400000011</v>
       </c>
       <c r="F25" s="6">
@@ -1361,11 +1454,15 @@
         <v>0.32605698047999992</v>
       </c>
       <c r="G25" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.67394301952000002</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I25" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0706333255927729</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>13</v>
       </c>
@@ -1389,8 +1486,12 @@
         <f>1-F26</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I26" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>13</v>
       </c>
@@ -1404,18 +1505,22 @@
         <v>0</v>
       </c>
       <c r="E27" s="11">
-        <f t="shared" ref="E27" si="11">1-D27</f>
+        <f t="shared" ref="E27" si="12">1-D27</f>
         <v>1</v>
       </c>
       <c r="F27" s="5">
         <v>0</v>
       </c>
       <c r="G27" s="11">
-        <f t="shared" ref="G27" si="12">1-F27</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" ref="G27" si="13">1-F27</f>
+        <v>1</v>
+      </c>
+      <c r="I27" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>13</v>
       </c>
@@ -1439,8 +1544,12 @@
         <f>1-F28</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I28" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>13</v>
       </c>
@@ -1466,8 +1575,12 @@
         <f>1-F29</f>
         <v>0.43059999999999998</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I29" s="28">
+        <f t="shared" si="2"/>
+        <v>1.9572727272727275</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>13</v>
       </c>
@@ -1482,7 +1595,7 @@
         <v>0.50700000000000001</v>
       </c>
       <c r="E30" s="11">
-        <f t="shared" ref="E30:E33" si="13">1-D30</f>
+        <f t="shared" ref="E30:E33" si="14">1-D30</f>
         <v>0.49299999999999999</v>
       </c>
       <c r="F30" s="6">
@@ -1490,11 +1603,15 @@
         <v>0.37010999999999999</v>
       </c>
       <c r="G30" s="11">
-        <f t="shared" ref="G30:G33" si="14">1-F30</f>
+        <f t="shared" ref="G30:G33" si="15">1-F30</f>
         <v>0.62989000000000006</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I30" s="28">
+        <f t="shared" si="2"/>
+        <v>1.2776673427991887</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>13</v>
       </c>
@@ -1509,7 +1626,7 @@
         <v>0.35489999999999999</v>
       </c>
       <c r="E31" s="11">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.64510000000000001</v>
       </c>
       <c r="F31" s="6">
@@ -1517,11 +1634,15 @@
         <v>0.259077</v>
       </c>
       <c r="G31" s="11">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0.740923</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I31" s="28">
+        <f t="shared" si="2"/>
+        <v>1.1485397612773214</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>13</v>
       </c>
@@ -1536,7 +1657,7 @@
         <v>0.24842999999999996</v>
       </c>
       <c r="E32" s="11">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.75157000000000007</v>
       </c>
       <c r="F32" s="6">
@@ -1544,11 +1665,15 @@
         <v>0.18135389999999996</v>
       </c>
       <c r="G32" s="11">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0.81864610000000004</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I32" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0892479742405896</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="7" t="s">
         <v>13</v>
       </c>
@@ -1563,7 +1688,7 @@
         <v>0.17390099999999997</v>
       </c>
       <c r="E33" s="13">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.82609900000000003</v>
       </c>
       <c r="F33" s="12">
@@ -1571,11 +1696,15 @@
         <v>0.12694772999999998</v>
       </c>
       <c r="G33" s="13">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0.87305227000000007</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I33" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0568373403187754</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="18" t="s">
         <v>19</v>
       </c>
@@ -1587,23 +1716,27 @@
         <v>0.83</v>
       </c>
       <c r="D34" s="21">
-        <f t="shared" ref="D34:G34" si="15">+D2</f>
+        <f t="shared" ref="D34:G34" si="16">+D2</f>
         <v>0</v>
       </c>
       <c r="E34" s="21">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
       <c r="F34" s="21">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="G34" s="22">
-        <f t="shared" si="15"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" si="16"/>
+        <v>1</v>
+      </c>
+      <c r="I34" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="18" t="s">
         <v>19</v>
       </c>
@@ -1611,27 +1744,31 @@
         <v>4</v>
       </c>
       <c r="C35" s="20">
-        <f t="shared" ref="C35:G41" si="16">+C3</f>
+        <f t="shared" ref="C35:G41" si="17">+C3</f>
         <v>0.83</v>
       </c>
       <c r="D35" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="E35" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="F35" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="G35" s="22">
-        <f t="shared" si="16"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="I35" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="18" t="s">
         <v>19</v>
       </c>
@@ -1639,27 +1776,31 @@
         <v>5</v>
       </c>
       <c r="C36" s="20">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.75</v>
       </c>
       <c r="D36" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="E36" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1</v>
       </c>
       <c r="F36" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="G36" s="22">
-        <f t="shared" si="16"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" si="17"/>
+        <v>1</v>
+      </c>
+      <c r="I36" s="28">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="18" t="s">
         <v>19</v>
       </c>
@@ -1667,27 +1808,31 @@
         <v>6</v>
       </c>
       <c r="C37" s="20">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.83</v>
       </c>
       <c r="D37" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.83</v>
       </c>
       <c r="E37" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.17000000000000004</v>
       </c>
       <c r="F37" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.62249999999999994</v>
       </c>
       <c r="G37" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.37750000000000006</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I37" s="28">
+        <f t="shared" si="2"/>
+        <v>2.2205882352941173</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="18" t="s">
         <v>19</v>
       </c>
@@ -1695,27 +1840,31 @@
         <v>7</v>
       </c>
       <c r="C38" s="20">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.96</v>
       </c>
       <c r="D38" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.79679999999999995</v>
       </c>
       <c r="E38" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.20320000000000005</v>
       </c>
       <c r="F38" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.59759999999999991</v>
       </c>
       <c r="G38" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.40240000000000009</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I38" s="28">
+        <f t="shared" si="2"/>
+        <v>1.9803149606299213</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="18" t="s">
         <v>19</v>
       </c>
@@ -1723,27 +1872,31 @@
         <v>8</v>
       </c>
       <c r="C39" s="20">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.61</v>
       </c>
       <c r="D39" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.48604799999999998</v>
       </c>
       <c r="E39" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.51395199999999996</v>
       </c>
       <c r="F39" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.36453599999999997</v>
       </c>
       <c r="G39" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.63546400000000003</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I39" s="28">
+        <f t="shared" si="2"/>
+        <v>1.2364267480231619</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="s">
         <v>19</v>
       </c>
@@ -1751,27 +1904,31 @@
         <v>9</v>
       </c>
       <c r="C40" s="20">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.61</v>
       </c>
       <c r="D40" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.29648927999999997</v>
       </c>
       <c r="E40" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.70351072000000003</v>
       </c>
       <c r="F40" s="21">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.22236695999999997</v>
       </c>
       <c r="G40" s="22">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.77763304</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="I40" s="28">
+        <f t="shared" si="2"/>
+        <v>1.1053606119889687</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>19</v>
       </c>
@@ -1779,28 +1936,38 @@
         <v>10</v>
       </c>
       <c r="C41" s="25">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.61</v>
       </c>
       <c r="D41" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.18085846079999998</v>
       </c>
       <c r="E41" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.81914153919999999</v>
       </c>
       <c r="F41" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.13564384559999998</v>
       </c>
       <c r="G41" s="27">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.86435615440000002</v>
+      </c>
+      <c r="I41" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0551975611493931</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f6b6dd5b-f02f-441a-99a0-162ac5060bd2}" enabled="0" method="" siteId="{f6b6dd5b-f02f-441a-99a0-162ac5060bd2}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>